<commit_message>
fix(parrillero-2.2): ronda de arreglos de la revisión final (4 mayores, 12 menores) + comida testigo del checklist del Paellero 2.2
- Comida testigo en TODOS los eventos: RD 1086/2020 art. 30.8.d («para eventos, cuando esta sea la
  actividad principal de la empresa»), verificado en el BOE consolidado; el «más de 40 personas» es el
  30.8.e. El checklist del Paellero 2.2 LIVE lo decía como condición doble: corregido y regenerado
  (cifras_caso_es.json idéntico).
- Tabla de cocción del manual y carta alineadas con la regla de 70 °C / «poco hecho» a petición;
  boda de ejemplo sin show de fuego (sigue a 42 €); landing con el escalado real (40-300 invitados).
- Ninguna cifra del caso movida. Gates verdes; Mac = VPS en los 13 ficheros.

Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-negocio-parrillero-asador-eventos/calculadora-pricing-eventos-parrillero.xlsx
+++ b/astro-site/public/dl/plan-negocio-parrillero-asador-eventos/calculadora-pricing-eventos-parrillero.xlsx
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B4" s="17" t="inlineStr">
         <is>
-          <t>Boda particular con show de fuego</t>
+          <t>Boda particular con cortes en mesa</t>
         </is>
       </c>
       <c r="C4" s="17" t="inlineStr">
@@ -2308,7 +2308,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C10" s="11" t="n">
         <v>3</v>
@@ -2436,7 +2436,7 @@
         </is>
       </c>
       <c r="B18" s="11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C18" s="11" t="n">
         <v>0</v>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>Boda particular con show de fuego</t>
+          <t>Boda particular con cortes en mesa</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="B34" s="11">
         <f>$B$10*$B$6</f>
-        <v>440.0</v>
+        <v>550.0</v>
       </c>
       <c r="C34" s="11">
         <f>$C$10*$C$6</f>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="B39" s="11">
         <f>$B$33+$B$34+$B$35+$B$36+$B$37+$B$38</f>
-        <v>2550.66</v>
+        <v>2660.66</v>
       </c>
       <c r="C39" s="11">
         <f>$C$33+$C$34+$C$35+$C$36+$C$37+$C$38</f>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="B40" s="11">
         <f>$B$39/$B$6</f>
-        <v>23.18781818181818</v>
+        <v>24.18781818181818</v>
       </c>
       <c r="C40" s="11">
         <f>$C$39/$C$6</f>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="B52" s="11">
         <f>$B$43-$B$39</f>
-        <v>2069.34</v>
+        <v>1959.3400000000001</v>
       </c>
       <c r="C52" s="11">
         <f>$C$43-$C$39</f>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="B53" s="16">
         <f>IF($B$43=0,0,$B$52/$B$43)</f>
-        <v>0.4479090909090909</v>
+        <v>0.42409956709956714</v>
       </c>
       <c r="C53" s="16">
         <f>IF($C$43=0,0,$C$52/$C$43)</f>
@@ -3177,12 +3177,12 @@
     <row r="60" ht="75" customHeight="1">
       <c r="A60" s="20" t="inlineStr">
         <is>
-          <t>Boda particular con show de fuego</t>
+          <t>Boda particular con cortes en mesa</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Particular, 110 invitados (la boda del caso del plan financiero), asado argentino de 500 g de carne cruda por invitado con cortes en mesa, bebida incluida y un suplemento de 2 € por invitado por el show de fuego. El precio con IVA es el que ve el particular; cobro en tres pagos (30 % al firmar, 40 % a siete días, 30 % a las 48 horas).</t>
+          <t>Particular, 110 invitados (la boda del caso del plan financiero), asado argentino de 500 g de carne cruda por invitado con cortes en mesa, bebida con vino incluida (5 €). Sin show: con él, súmale de 8 a 15 € por invitado. El precio con IVA es el que ve el particular; cobro en tres pagos (30 % al firmar, 40 % a siete días, 30 % a las 48 horas).</t>
         </is>
       </c>
     </row>
@@ -3408,7 +3408,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Versión 2.2 · septiembre 2026 · aichef.pro/plan-negocio-parrillero-asador-eventos · info@aichef.pro</t>
+          <t>Versión 2.2 · octubre 2026 · aichef.pro/plan-negocio-parrillero-asador-eventos · info@aichef.pro</t>
         </is>
       </c>
     </row>

</xml_diff>